<commit_message>
small EBMKF_ta4 edits, removed unnecessary GAM_AR1 baseline adjustment
</commit_message>
<xml_diff>
--- a/Common_Data/toyKFmodelData9_ext.xlsx
+++ b/Common_Data/toyKFmodelData9_ext.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/JohnMatthew/Downloads/Thorne_15_codefigurestats/Common_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{88DEFCA1-D87D-4A43-8302-BE298EE7F39F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{50995EC3-783F-6148-B84C-311E8A52D704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10780" yWindow="600" windowWidth="35840" windowHeight="20920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3560" yWindow="600" windowWidth="35860" windowHeight="20120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="toyKFmodelData8c" sheetId="1" r:id="rId1"/>

</xml_diff>